<commit_message>
Energypedia: wezwanie „Dodaj do preferowanych źródeł” w Google (makiety, architektura, wymagania techniczne)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rv6z9UcN5eHj71s4nzprHT
</commit_message>
<xml_diff>
--- a/docs/energypedia/mapa/Energypedia_mapa_tematow.xlsx
+++ b/docs/energypedia/mapa/Energypedia_mapa_tematow.xlsx
@@ -25,7 +25,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Kanibalizacja'!$A$1:$D$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Regiony'!$A$1:$E$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Taksonomia'!$A$1:$C$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Technika SEO i GEO'!$A$1:$B$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Technika SEO i GEO'!$A$1:$B$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24042,7 +24042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -24268,53 +24268,65 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>E-E-A-T</t>
+          <t>Preferowane źródła Google</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Strony: Jak pracujemy, Jak zarabiamy, Redakcja, Sprostowania, strony autorów z biogramem; podpis autora i recenzenta przy każdej publikacji.</t>
+          <t>Wezwanie „Dodaj do preferowanych źródeł” (link https://www.google.com/preferences/source?q=energypedia.pl lub oficjalny przycisk z Search Central) pod artykułami, w panelu „Więcej” i w stopce; pomiar kliknięć; regularne newsy, bo funkcja działa w sekcji „Najważniejsze artykuły”. [DO WERYFIKACJI: wytyczne i kod przycisku]</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Google News i Discover</t>
+          <t>E-E-A-T</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Zgłoszenie w Google Publisher Center; obrazy co najmniej 1200 px szerokości; tytuły bez clickbaitu; jasna data publikacji.</t>
+          <t>Strony: Jak pracujemy, Jak zarabiamy, Redakcja, Sprostowania, strony autorów z biogramem; podpis autora i recenzenta przy każdej publikacji.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Kanały</t>
+          <t>Google News i Discover</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>RSS/Atom: całość, obszary, trackery; API danych Barometru; wykresy do osadzenia z linkiem zwrotnym.</t>
+          <t>Zgłoszenie w Google Publisher Center; obrazy co najmniej 1200 px szerokości; tytuły bez clickbaitu; jasna data publikacji.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
+          <t>Kanały</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>RSS/Atom: całość, obszary, trackery; API danych Barometru; wykresy do osadzenia z linkiem zwrotnym.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
           <t>Język</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>ZASADY_Energypedia.md: poprawna polszczyzna, bez długiego myślnika, typografia liczb i dat; lang="pl" w HTML.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B22"/>
+  <autoFilter ref="A1:B23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Energypedia: asystent AI w MVP, temat miesiąca o zmianie sprzedawcy
Asystent „Zapytaj Energypedię” dopisany do zakresu MVP (plan, architektura
ADR-13, biznesplan), temat miesiąca w mapie tematów i propozycji strony głównej.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rv6z9UcN5eHj71s4nzprHT
</commit_message>
<xml_diff>
--- a/docs/energypedia/mapa/Energypedia_mapa_tematow.xlsx
+++ b/docs/energypedia/mapa/Energypedia_mapa_tematow.xlsx
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Obszary'!$A$1:$H$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Publikacje MVP'!$A$1:$T$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Publikacje MVP'!$A$1:$T$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Hasła'!$A$1:$H$301</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Pytania long tail'!$A$1:$F$201</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Kanibalizacja'!$A$1:$D$12</definedName>
@@ -487,7 +487,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Publikacje MVP – 74 publikacji do 31.12.2026 r.: 5 przewodników, 2 trackery, 20 artykułów i porównań, 5 analiz, 25 poradników, 5 wzorów pism, katalog: 5 sprzedawców z urzędu i 5 operatorów sieci ze stronami zbiorczymi.</t>
+          <t>Publikacje MVP – 75 publikacji do 31.12.2026 r.: 5 przewodników, 2 trackery, 20 artykułów i porównań, 5 analiz, 25 poradników, 5 wzorów pism, katalog: 5 sprzedawców z urzędu i 5 operatorów sieci ze stronami zbiorczymi.</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>25</v>
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T75"/>
+  <dimension ref="A1:T76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1955,32 +1955,32 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>przewodnik</t>
+          <t>temat miesiąca</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Rachunek za prąd i opłaty</t>
+          <t>Umowy i zmiana sprzedawcy</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Rachunek za prąd: z czego się składa, ile płacimy i jak go obniżyć</t>
+          <t>Zmiana sprzedawcy prądu 2027: kiedy wypowiedzieć umowę</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>rachunek za prąd</t>
+          <t>kiedy wypowiedzieć umowę na prąd</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>jak czytać rachunek za prąd; opłaty na rachunku za prąd; dlaczego rachunek za prąd jest wysoki; rachunek za prąd 2026</t>
+          <t>wypowiedzenie umowy na prąd termin; zmiana sprzedawcy od 1 stycznia 2027; okres wypowiedzenia umowy na prąd; czy mogę zerwać umowę na prąd na czas określony; zmiana sprzedawcy prądu 2027</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>informacyjna</t>
+          <t>informacyjna i transakcyjna</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1990,42 +1990,42 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/rachunek-za-prad</t>
+          <t>/temat/zmiana-sprzedawcy-2027</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/rachunek-za-prad</t>
+          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>tabela</t>
+          <t>lista</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Article + BreadcrumbList + FAQPage</t>
+          <t>CollectionPage + Article + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M11" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q11" s="4" t="n">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="R11" s="4" t="inlineStr">
         <is>
-          <t>styczeń–luty (rozliczenia), grudzień</t>
+          <t>listopad–styczeń (koniec umów rocznych, decyzja URE)</t>
         </is>
       </c>
       <c r="S11" s="4" t="inlineStr">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: URE wskazuje pytanie o opłaty na rachunku jako jedno z najczęściej zadawanych (FAQ URE); koniec mrożenia cen od 1.01.2026.</t>
+          <t>Brak wolumenu. Sygnał: 45 891 zmian sprzedawcy prądu w I półroczu 2026 r. (URE).</t>
         </is>
       </c>
     </row>
@@ -2050,27 +2050,27 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Umowy i zmiana sprzedawcy</t>
+          <t>Rachunek za prąd i opłaty</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Zmiana sprzedawcy prądu: prawa odbiorcy, umowy i pułapki</t>
+          <t>Rachunek za prąd: z czego się składa, ile płacimy i jak go obniżyć</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>zmiana sprzedawcy prądu</t>
+          <t>rachunek za prąd</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>jak zmienić sprzedawcę prądu; czy opłaca się zmienić sprzedawcę prądu; zmiana sprzedawcy prądu w 24 godziny</t>
+          <t>jak czytać rachunek za prąd; opłaty na rachunku za prąd; dlaczego rachunek za prąd jest wysoki; rachunek za prąd 2026</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>informacyjna i transakcyjna</t>
+          <t>informacyjna</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -2080,17 +2080,17 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
+          <t>/przewodniki/rachunek-za-prad</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
+          <t>/przewodniki/rachunek-za-prad</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>tabela</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
@@ -2099,13 +2099,13 @@
         </is>
       </c>
       <c r="M12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>2</v>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="R12" s="4" t="inlineStr">
         <is>
-          <t>cały rok, wzrost przy podwyżkach</t>
+          <t>styczeń–luty (rozliczenia), grudzień</t>
         </is>
       </c>
       <c r="S12" s="4" t="inlineStr">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="T12" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: 45 891 zmian sprzedawcy prądu w I półroczu 2026 r. (URE).</t>
+          <t>Brak wolumenu. Sygnał: URE wskazuje pytanie o opłaty na rachunku jako jedno z najczęściej zadawanych (FAQ URE); koniec mrożenia cen od 1.01.2026.</t>
         </is>
       </c>
     </row>
@@ -2140,47 +2140,47 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Energia dla firm</t>
+          <t>Umowy i zmiana sprzedawcy</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Prąd dla firm: ceny, umowy i zakupy energii</t>
+          <t>Zmiana sprzedawcy prądu: prawa odbiorcy, umowy i pułapki</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>prąd dla firm</t>
+          <t>zmiana sprzedawcy prądu</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>ceny prądu dla firm 2026; cena prądu dla firm za kWh; umowa na prąd dla firmy; ile kosztuje prąd w firmie</t>
+          <t>jak zmienić sprzedawcę prądu; czy opłaca się zmienić sprzedawcę prądu; zmiana sprzedawcy prądu w 24 godziny</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>informacyjna i porównawcza</t>
+          <t>informacyjna i transakcyjna</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>mikro, msp, duże</t>
+          <t>dom, mikro</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/prad-dla-firm</t>
+          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/prad-dla-firm</t>
+          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>tabela</t>
+          <t>lista</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="R13" s="4" t="inlineStr">
         <is>
-          <t>IV kwartał (kontraktacja na kolejny rok)</t>
+          <t>cały rok, wzrost przy podwyżkach</t>
         </is>
       </c>
       <c r="S13" s="4" t="inlineStr">
@@ -2215,7 +2215,7 @@
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
+          <t>Brak wolumenu. Sygnał: 45 891 zmian sprzedawcy prądu w I półroczu 2026 r. (URE).</t>
         </is>
       </c>
     </row>
@@ -2225,52 +2225,52 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>artykuł</t>
+          <t>przewodnik</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Rachunek za prąd i opłaty</t>
+          <t>Energia dla firm</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Dlaczego rachunek za prąd rośnie, choć prąd na giełdzie tanieje</t>
+          <t>Prąd dla firm: ceny, umowy i zakupy energii</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>dlaczego prąd jest drogi</t>
+          <t>prąd dla firm</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>dlaczego rachunek za prąd wzrósł; ceny prądu na giełdzie a rachunek</t>
+          <t>ceny prądu dla firm 2026; cena prądu dla firm za kWh; umowa na prąd dla firmy; ile kosztuje prąd w firmie</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>informacyjna</t>
+          <t>informacyjna i porównawcza</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>dom, mikro</t>
+          <t>mikro, msp, duże</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/dlaczego-rachunek-za-prad-rosnie</t>
+          <t>/przewodniki/prad-dla-firm</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/rachunek-za-prad</t>
+          <t>/przewodniki/prad-dla-firm</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>akapit</t>
+          <t>tabela</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
@@ -2279,10 +2279,10 @@
         </is>
       </c>
       <c r="M14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N14" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="N14" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="O14" s="4" t="n">
         <v>3</v>
@@ -2295,7 +2295,7 @@
       </c>
       <c r="R14" s="4" t="inlineStr">
         <is>
-          <t>po decyzji URE</t>
+          <t>IV kwartał (kontraktacja na kolejny rok)</t>
         </is>
       </c>
       <c r="S14" s="4" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="T14" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: URE wskazuje pytanie o opłaty na rachunku jako jedno z najczęściej zadawanych (FAQ URE); koniec mrożenia cen od 1.01.2026.</t>
+          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
         </is>
       </c>
     </row>
@@ -2320,22 +2320,22 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Taryfy i ceny prądu</t>
+          <t>Rachunek za prąd i opłaty</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Taryfa dynamiczna: dla kogo, jakie ryzyko i ile można zaoszczędzić</t>
+          <t>Dlaczego rachunek za prąd rośnie, choć prąd na giełdzie tanieje</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>taryfa dynamiczna</t>
+          <t>dlaczego prąd jest drogi</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>ceny dynamiczne prądu; umowa z ceną dynamiczną; czy taryfa dynamiczna się opłaca</t>
+          <t>dlaczego rachunek za prąd wzrósł; ceny prądu na giełdzie a rachunek</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -2350,12 +2350,12 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/taryfa-dynamiczna</t>
+          <t>/poradniki/dlaczego-rachunek-za-prad-rosnie</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/ceny-pradu</t>
+          <t>/przewodniki/rachunek-za-prad</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
@@ -2369,10 +2369,10 @@
         </is>
       </c>
       <c r="M15" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N15" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="N15" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="O15" s="4" t="n">
         <v>3</v>
@@ -2385,17 +2385,17 @@
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>cały rok</t>
+          <t>po decyzji URE</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 20.11)</t>
         </is>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: 4 836 gospodarstw domowych z ceną dynamiczną na koniec 2025 r. wobec 135 rok wcześniej; liczniki zdalnego odczytu u 48% odbiorców (URE).</t>
+          <t>Brak wolumenu. Sygnał: URE wskazuje pytanie o opłaty na rachunku jako jedno z najczęściej zadawanych (FAQ URE); koniec mrożenia cen od 1.01.2026.</t>
         </is>
       </c>
     </row>
@@ -2410,47 +2410,47 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Energia dla firm</t>
+          <t>Taryfy i ceny prądu</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Ile kosztuje prąd w małej firmie: przykłady dla 5 branż</t>
+          <t>Taryfa dynamiczna: dla kogo, jakie ryzyko i ile można zaoszczędzić</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>ile kosztuje prąd w firmie</t>
+          <t>taryfa dynamiczna</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>koszt prądu w sklepie; koszt prądu w piekarni; koszt prądu w gastronomii</t>
+          <t>ceny dynamiczne prądu; umowa z ceną dynamiczną; czy taryfa dynamiczna się opłaca</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>porównawcza</t>
+          <t>informacyjna</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>mikro</t>
+          <t>dom, mikro</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/ile-kosztuje-prad-w-firmie</t>
+          <t>/poradniki/taryfa-dynamiczna</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/prad-dla-firm</t>
+          <t>/przewodniki/ceny-pradu</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>tabela</t>
+          <t>akapit</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>IV kwartał</t>
+          <t>cały rok</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="T16" s="4" t="inlineStr">
         <is>
-          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
+          <t>Brak wolumenu. Sygnał: 4 836 gospodarstw domowych z ceną dynamiczną na koniec 2025 r. wobec 135 rok wcześniej; liczniki zdalnego odczytu u 48% odbiorców (URE).</t>
         </is>
       </c>
     </row>
@@ -2500,22 +2500,22 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Magazyny, pompy ciepła, samochody elektryczne</t>
+          <t>Energia dla firm</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Pompa ciepła a rachunek za prąd: ile naprawdę kosztuje ogrzewanie</t>
+          <t>Ile kosztuje prąd w małej firmie: przykłady dla 5 branż</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>pompa ciepła zużycie prądu</t>
+          <t>ile kosztuje prąd w firmie</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>ile prądu zużywa pompa ciepła; koszt ogrzewania pompą ciepła; taryfa dla pompy ciepła; jak działa pompa ciepła; ile kosztuje pompa ciepła</t>
+          <t>koszt prądu w sklepie; koszt prądu w piekarni; koszt prądu w gastronomii</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -2525,17 +2525,17 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>dom</t>
+          <t>mikro</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/pompa-ciepla-rachunek-za-prad</t>
+          <t>/poradniki/ile-kosztuje-prad-w-firmie</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/magazyn-energii</t>
+          <t>/przewodniki/prad-dla-firm</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
@@ -2549,33 +2549,33 @@
         </is>
       </c>
       <c r="M17" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N17" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="N17" s="4" t="n">
+      <c r="O17" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P17" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="O17" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P17" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="Q17" s="4" t="n">
         <v>36</v>
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>szczyt XII–II, publikacja do połowy XI</t>
+          <t>IV kwartał</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 2 (do 4.12)</t>
         </is>
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>Wolumen: „pompa ciepła” ok. 60 500/mies., w styczniu ok. 135 000, szczyt XII–II; „jak działa pompa ciepła” ok. 5 400; „ile kosztuje pompa ciepła” ok. 2 900 (widzialnosc.co.pl, ok. IV 2026). Sygnał przeciwny: zapytania ofertowe o pompy ciepła −51% r/r I–VIII 2026 (Oferteo).</t>
+          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
         </is>
       </c>
     </row>
@@ -2590,47 +2590,47 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Umowy i zmiana sprzedawcy</t>
+          <t>Magazyny, pompy ciepła, samochody elektryczne</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Akwizytorzy energii: jak rozpoznać nieuczciwą ofertę</t>
+          <t>Pompa ciepła a rachunek za prąd: ile naprawdę kosztuje ogrzewanie</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>akwizytor prąd</t>
+          <t>pompa ciepła zużycie prądu</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>akwizytor energii oszustwo; umowa z akwizytorem prąd; jak odstąpić od umowy z akwizytorem</t>
+          <t>ile prądu zużywa pompa ciepła; koszt ogrzewania pompą ciepła; taryfa dla pompy ciepła; jak działa pompa ciepła; ile kosztuje pompa ciepła</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>informacyjna</t>
+          <t>porównawcza</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>dom, mikro</t>
+          <t>dom</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/akwizytorzy-energii</t>
+          <t>/poradniki/pompa-ciepla-rachunek-za-prad</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
+          <t>/przewodniki/magazyn-energii</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>tabela</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -2639,23 +2639,23 @@
         </is>
       </c>
       <c r="M18" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N18" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="N18" s="4" t="n">
+      <c r="O18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P18" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="O18" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="P18" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>36</v>
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>cały rok</t>
+          <t>szczyt XII–II, publikacja do połowy XI</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="T18" s="4" t="inlineStr">
         <is>
-          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
+          <t>Wolumen: „pompa ciepła” ok. 60 500/mies., w styczniu ok. 135 000, szczyt XII–II; „jak działa pompa ciepła” ok. 5 400; „ile kosztuje pompa ciepła” ok. 2 900 (widzialnosc.co.pl, ok. IV 2026). Sygnał przeciwny: zapytania ofertowe o pompy ciepła −51% r/r I–VIII 2026 (Oferteo).</t>
         </is>
       </c>
     </row>
@@ -2675,7 +2675,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>poradnik</t>
+          <t>artykuł</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -2685,22 +2685,22 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Jak zmienić sprzedawcę prądu krok po kroku</t>
+          <t>Akwizytorzy energii: jak rozpoznać nieuczciwą ofertę</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>jak zmienić sprzedawcę prądu</t>
+          <t>akwizytor prąd</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>zmiana sprzedawcy prądu krok po kroku; dokumenty do zmiany sprzedawcy</t>
+          <t>akwizytor energii oszustwo; umowa z akwizytorem prąd; jak odstąpić od umowy z akwizytorem</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>poradnikowa (jak)</t>
+          <t>informacyjna</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -2710,7 +2710,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/jak-zmienic-sprzedawce-pradu</t>
+          <t>/poradniki/akwizytorzy-energii</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -2725,7 +2725,7 @@
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Article (HowTo jako struktura treści) + BreadcrumbList + FAQPage</t>
+          <t>Article + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M19" s="4" t="n">
@@ -2755,7 +2755,7 @@
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: 45 891 zmian sprzedawcy prądu w I półroczu 2026 r. (URE).</t>
+          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
         </is>
       </c>
     </row>
@@ -2770,22 +2770,22 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Rachunek za prąd i opłaty</t>
+          <t>Umowy i zmiana sprzedawcy</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Jak czytać rachunek za prąd: pozycja po pozycji</t>
+          <t>Jak zmienić sprzedawcę prądu krok po kroku</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>jak czytać rachunek za prąd</t>
+          <t>jak zmienić sprzedawcę prądu</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>opłaty na rachunku za prąd wyjaśnienie; faktura za prąd</t>
+          <t>zmiana sprzedawcy prądu krok po kroku; dokumenty do zmiany sprzedawcy</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -2800,12 +2800,12 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/jak-czytac-rachunek-za-prad</t>
+          <t>/poradniki/jak-zmienic-sprzedawce-pradu</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/rachunek-za-prad</t>
+          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
@@ -2819,13 +2819,13 @@
         </is>
       </c>
       <c r="M20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N20" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O20" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>2</v>
@@ -2845,7 +2845,7 @@
       </c>
       <c r="T20" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: URE wskazuje pytanie o opłaty na rachunku jako jedno z najczęściej zadawanych (FAQ URE); koniec mrożenia cen od 1.01.2026.</t>
+          <t>Brak wolumenu. Sygnał: 45 891 zmian sprzedawcy prądu w I półroczu 2026 r. (URE).</t>
         </is>
       </c>
     </row>
@@ -2860,22 +2860,22 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Prosumenci i OZE</t>
+          <t>Rachunek za prąd i opłaty</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Jak ubiegać się o dotację do magazynu energii i fotowoltaiki</t>
+          <t>Jak czytać rachunek za prąd: pozycja po pozycji</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>dotacja do magazynu energii</t>
+          <t>jak czytać rachunek za prąd</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Przydomowe Magazyny Energii (PME2) [DO WERYFIKACJI warunki NFOŚiGW]; dofinansowanie magazynu energii; dotacja do fotowoltaiki; ulga termomodernizacyjna fotowoltaika</t>
+          <t>opłaty na rachunku za prąd wyjaśnienie; faktura za prąd</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -2890,12 +2890,12 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/dotacja-do-magazynu-energii</t>
+          <t>/poradniki/jak-czytac-rachunek-za-prad</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/fotowoltaika</t>
+          <t>/przewodniki/rachunek-za-prad</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
@@ -2912,13 +2912,13 @@
         <v>3</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O21" s="4" t="n">
         <v>2</v>
       </c>
       <c r="P21" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q21" s="4" t="n">
         <v>36</v>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>Wolumen: „magazyn energii” ok. 33 100/mies., wzrost ponad 50% r/r, KD 3/100; „magazyn energii 10kw” 12 100; „magazyn energii 20kwh” 6 600 (agencja widzialnosc.co.pl, Planer słów kluczowych lub DataForSEO, ok. IV 2026). Sygnał: 60% wniosków w Mój Prąd 6.0 dotyczyło magazynów; nabór PME2 od 20.10.2026 (NFOŚiGW, za gramwzielone.pl). | Sygnał: Mój Prąd 6.0 – ponad 121 tys. wniosków (nabór zakończony 12.09.2025); PME2 od 20.10.2026, budżet 1 mld zł (NFOŚiGW, za mediami). [DO WERYFIKACJI warunki programów] | Wolumen: „fotowoltaika” ok. 90 500/mies. (agencjaecho.pl, ok. 2026; podobnie widzialnosc.co.pl). Polska 3. na świecie pod względem zainteresowania fotowoltaiką w Google w latach 2020–2025 (komunikat prasowy, VI 2026, metodologia nieopublikowana).</t>
+          <t>Brak wolumenu. Sygnał: URE wskazuje pytanie o opłaty na rachunku jako jedno z najczęściej zadawanych (FAQ URE); koniec mrożenia cen od 1.01.2026.</t>
         </is>
       </c>
     </row>
@@ -2950,22 +2950,22 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Magazyny, pompy ciepła, samochody elektryczne</t>
+          <t>Prosumenci i OZE</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Jak dobrać magazyn energii do instalacji fotowoltaicznej</t>
+          <t>Jak ubiegać się o dotację do magazynu energii i fotowoltaiki</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>jaki magazyn energii wybrać</t>
+          <t>dotacja do magazynu energii</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>pojemność magazynu energii dla domu; magazyn energii kWh; magazyn energii 10 kW</t>
+          <t>Przydomowe Magazyny Energii (PME2) [DO WERYFIKACJI warunki NFOŚiGW]; dofinansowanie magazynu energii; dotacja do fotowoltaiki; ulga termomodernizacyjna fotowoltaika</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -2980,12 +2980,12 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/jaki-magazyn-energii-wybrac</t>
+          <t>/poradniki/dotacja-do-magazynu-energii</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/magazyn-energii</t>
+          <t>/przewodniki/fotowoltaika</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
@@ -3005,10 +3005,10 @@
         <v>2</v>
       </c>
       <c r="O22" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P22" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="Q22" s="4" t="n">
         <v>36</v>
@@ -3025,7 +3025,7 @@
       </c>
       <c r="T22" s="4" t="inlineStr">
         <is>
-          <t>Wolumen: „magazyn energii” ok. 33 100/mies., wzrost ponad 50% r/r, KD 3/100; „magazyn energii 10kw” 12 100; „magazyn energii 20kwh” 6 600 (agencja widzialnosc.co.pl, Planer słów kluczowych lub DataForSEO, ok. IV 2026). Sygnał: 60% wniosków w Mój Prąd 6.0 dotyczyło magazynów; nabór PME2 od 20.10.2026 (NFOŚiGW, za gramwzielone.pl).</t>
+          <t>Wolumen: „magazyn energii” ok. 33 100/mies., wzrost ponad 50% r/r, KD 3/100; „magazyn energii 10kw” 12 100; „magazyn energii 20kwh” 6 600 (agencja widzialnosc.co.pl, Planer słów kluczowych lub DataForSEO, ok. IV 2026). Sygnał: 60% wniosków w Mój Prąd 6.0 dotyczyło magazynów; nabór PME2 od 20.10.2026 (NFOŚiGW, za gramwzielone.pl). | Sygnał: Mój Prąd 6.0 – ponad 121 tys. wniosków (nabór zakończony 12.09.2025); PME2 od 20.10.2026, budżet 1 mld zł (NFOŚiGW, za mediami). [DO WERYFIKACJI warunki programów] | Wolumen: „fotowoltaika” ok. 90 500/mies. (agencjaecho.pl, ok. 2026; podobnie widzialnosc.co.pl). Polska 3. na świecie pod względem zainteresowania fotowoltaiką w Google w latach 2020–2025 (komunikat prasowy, VI 2026, metodologia nieopublikowana).</t>
         </is>
       </c>
     </row>
@@ -3035,32 +3035,32 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>katalog</t>
+          <t>poradnik</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Umowy i zmiana sprzedawcy</t>
+          <t>Magazyny, pompy ciepła, samochody elektryczne</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Sprzedawcy prądu w Polsce: kto jest Twoim sprzedawcą z urzędu</t>
+          <t>Jak dobrać magazyn energii do instalacji fotowoltaicznej</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>sprzedawcy prądu</t>
+          <t>jaki magazyn energii wybrać</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>sprzedawca z urzędu; lista sprzedawców energii; jak sprawdzić sprzedawcę prądu</t>
+          <t>pojemność magazynu energii dla domu; magazyn energii kWh; magazyn energii 10 kW</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>informacyjna i nawigacyjna</t>
+          <t>poradnikowa (jak)</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -3070,29 +3070,29 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>/sprzedawcy</t>
+          <t>/poradniki/jaki-magazyn-energii-wybrac</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
+          <t>/przewodniki/magazyn-energii</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>tabela</t>
+          <t>lista</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>CollectionPage + ItemList + BreadcrumbList</t>
+          <t>Article (HowTo jako struktura treści) + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M23" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N23" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="N23" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="O23" s="4" t="n">
         <v>3</v>
@@ -3105,17 +3105,17 @@
       </c>
       <c r="R23" s="4" t="inlineStr">
         <is>
-          <t>grudzień–styczeń (taryfy)</t>
+          <t>cały rok</t>
         </is>
       </c>
       <c r="S23" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 20.11)</t>
         </is>
       </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: 45 891 zmian sprzedawcy prądu w I półroczu 2026 r. (URE).</t>
+          <t>Wolumen: „magazyn energii” ok. 33 100/mies., wzrost ponad 50% r/r, KD 3/100; „magazyn energii 10kw” 12 100; „magazyn energii 20kwh” 6 600 (agencja widzialnosc.co.pl, Planer słów kluczowych lub DataForSEO, ok. IV 2026). Sygnał: 60% wniosków w Mój Prąd 6.0 dotyczyło magazynów; nabór PME2 od 20.10.2026 (NFOŚiGW, za gramwzielone.pl).</t>
         </is>
       </c>
     </row>
@@ -3125,47 +3125,47 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>artykuł</t>
+          <t>katalog</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Energia dla firm</t>
+          <t>Umowy i zmiana sprzedawcy</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Cena stała czy indeksowana: jak firma powinna kupować prąd</t>
+          <t>Sprzedawcy prądu w Polsce: kto jest Twoim sprzedawcą z urzędu</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>cena stała czy indeksowana</t>
+          <t>sprzedawcy prądu</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>umowa z ceną indeksowaną; cena prądu indeksowana do TGE; zakup energii dla firm</t>
+          <t>sprzedawca z urzędu; lista sprzedawców energii; jak sprawdzić sprzedawcę prądu</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>porównawcza</t>
+          <t>informacyjna i nawigacyjna</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>msp, duże</t>
+          <t>dom, mikro</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/cena-stala-czy-indeksowana</t>
+          <t>/sprzedawcy</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/prad-dla-firm</t>
+          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
@@ -3175,11 +3175,11 @@
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>Article + BreadcrumbList + FAQPage</t>
+          <t>CollectionPage + ItemList + BreadcrumbList</t>
         </is>
       </c>
       <c r="M24" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N24" s="4" t="n">
         <v>3</v>
@@ -3188,24 +3188,24 @@
         <v>3</v>
       </c>
       <c r="P24" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q24" s="4" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="R24" s="4" t="inlineStr">
         <is>
-          <t>IV kwartał</t>
+          <t>grudzień–styczeń (taryfy)</t>
         </is>
       </c>
       <c r="S24" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 2 (do 4.12)</t>
         </is>
       </c>
       <c r="T24" s="4" t="inlineStr">
         <is>
-          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
+          <t>Brak wolumenu. Sygnał: 45 891 zmian sprzedawcy prądu w I półroczu 2026 r. (URE).</t>
         </is>
       </c>
     </row>
@@ -3215,43 +3215,47 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>analiza</t>
+          <t>artykuł</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Rynek i system energetyczny</t>
+          <t>Energia dla firm</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Barometr Rynku Energii #1: grudzień 2026</t>
+          <t>Cena stała czy indeksowana: jak firma powinna kupować prąd</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>ceny prądu na giełdzie</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr"/>
+          <t>cena stała czy indeksowana</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>umowa z ceną indeksowaną; cena prądu indeksowana do TGE; zakup energii dla firm</t>
+        </is>
+      </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>informacyjna (dane)</t>
+          <t>porównawcza</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>wszyscy, media</t>
+          <t>msp, duże</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>/dane/barometr-rynku/2026-12</t>
+          <t>/poradniki/cena-stala-czy-indeksowana</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/rynek-energii</t>
+          <t>/przewodniki/prad-dla-firm</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
@@ -3261,7 +3265,7 @@
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>Article + Dataset + BreadcrumbList</t>
+          <t>Article + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M25" s="4" t="n">
@@ -3281,12 +3285,12 @@
       </c>
       <c r="R25" s="4" t="inlineStr">
         <is>
-          <t>co miesiąc</t>
+          <t>IV kwartał</t>
         </is>
       </c>
       <c r="S25" s="4" t="inlineStr">
         <is>
-          <t>Tydzień startu</t>
+          <t>Fala 1 (do 20.11)</t>
         </is>
       </c>
       <c r="T25" s="4" t="inlineStr">
@@ -3306,17 +3310,17 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Taryfy i ceny prądu</t>
+          <t>Rynek i system energetyczny</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Temperatura rachunku: ile kosztuje rok prądu u typowego odbiorcy</t>
+          <t>Barometr Rynku Energii #1: grudzień 2026</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>koszt prądu rocznie</t>
+          <t>ceny prądu na giełdzie</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
@@ -3332,12 +3336,12 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>/dane/temperatura-rachunku</t>
+          <t>/dane/barometr-rynku/2026-12</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/ceny-pradu</t>
+          <t>/przewodniki/rynek-energii</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
@@ -3397,12 +3401,12 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Taryfy 2027 a 2026: porównanie według operatorów sieci</t>
+          <t>Temperatura rachunku: ile kosztuje rok prądu u typowego odbiorcy</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>taryfy dystrybucyjne 2027</t>
+          <t>koszt prądu rocznie</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr"/>
@@ -3418,7 +3422,7 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>/analizy/taryfy-2027-a-2026-porownanie</t>
+          <t>/dane/temperatura-rachunku</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -3453,7 +3457,7 @@
       </c>
       <c r="R27" s="4" t="inlineStr">
         <is>
-          <t>grudzień</t>
+          <t>co miesiąc</t>
         </is>
       </c>
       <c r="S27" s="4" t="inlineStr">
@@ -3478,17 +3482,17 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Rynek i system energetyczny</t>
+          <t>Taryfy i ceny prądu</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Godziny z ujemnymi cenami prądu w 2026 r.</t>
+          <t>Taryfy 2027 a 2026: porównanie według operatorów sieci</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>ujemne ceny prądu 2026</t>
+          <t>taryfy dystrybucyjne 2027</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
@@ -3504,12 +3508,12 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>/analizy/ujemne-ceny-pradu-2026</t>
+          <t>/analizy/taryfy-2027-a-2026-porownanie</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/rynek-energii</t>
+          <t>/przewodniki/ceny-pradu</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr">
@@ -3564,17 +3568,17 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Rachunek za prąd i opłaty</t>
+          <t>Rynek i system energetyczny</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Barometr Odbiorców Energii #0: jak Polacy i firmy oceniają rachunki</t>
+          <t>Godziny z ujemnymi cenami prądu w 2026 r.</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>badanie rachunki za prąd</t>
+          <t>ujemne ceny prądu 2026</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr"/>
@@ -3590,12 +3594,12 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>/dane/barometr-odbiorcow/2026-4</t>
+          <t>/analizy/ujemne-ceny-pradu-2026</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/rachunek-za-prad</t>
+          <t>/przewodniki/rynek-energii</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr">
@@ -3625,7 +3629,7 @@
       </c>
       <c r="R29" s="4" t="inlineStr">
         <is>
-          <t>kwartalnie</t>
+          <t>grudzień</t>
         </is>
       </c>
       <c r="S29" s="4" t="inlineStr">
@@ -3645,57 +3649,53 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>poradnik</t>
+          <t>analiza</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Energia dla firm</t>
+          <t>Rachunek za prąd i opłaty</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Jak przygotować zapytanie ofertowe na energię dla firmy</t>
+          <t>Barometr Odbiorców Energii #0: jak Polacy i firmy oceniają rachunki</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>zapytanie ofertowe energia</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>jak kupić prąd dla firmy; oferty prądu dla firm</t>
-        </is>
-      </c>
+          <t>badanie rachunki za prąd</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr"/>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>poradnikowa (jak)</t>
+          <t>informacyjna (dane)</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>msp</t>
+          <t>wszyscy, media</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/zapytanie-ofertowe-energia</t>
+          <t>/dane/barometr-odbiorcow/2026-4</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/prad-dla-firm</t>
+          <t>/przewodniki/rachunek-za-prad</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>tabela</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Article (HowTo jako struktura treści) + BreadcrumbList + FAQPage</t>
+          <t>Article + Dataset + BreadcrumbList</t>
         </is>
       </c>
       <c r="M30" s="4" t="n">
@@ -3715,12 +3715,12 @@
       </c>
       <c r="R30" s="4" t="inlineStr">
         <is>
-          <t>cały rok</t>
+          <t>kwartalnie</t>
         </is>
       </c>
       <c r="S30" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Tydzień startu</t>
         </is>
       </c>
       <c r="T30" s="4" t="inlineStr">
@@ -3735,77 +3735,77 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>artykuł</t>
+          <t>poradnik</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Rachunek za prąd i opłaty</t>
+          <t>Energia dla firm</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Opłata mocowa: kto płaci, ile i dlaczego</t>
+          <t>Jak przygotować zapytanie ofertowe na energię dla firmy</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>opłata mocowa</t>
+          <t>zapytanie ofertowe energia</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>opłata mocowa 2026; opłata mocowa co to; opłata mocowa stawki</t>
+          <t>jak kupić prąd dla firmy; oferty prądu dla firm</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>porównawcza</t>
+          <t>poradnikowa (jak)</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>wszyscy</t>
+          <t>msp</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/oplata-mocowa</t>
+          <t>/poradniki/zapytanie-ofertowe-energia</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/rachunek-za-prad</t>
+          <t>/przewodniki/prad-dla-firm</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>tabela</t>
+          <t>lista</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>Article + BreadcrumbList + FAQPage</t>
+          <t>Article (HowTo jako struktura treści) + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N31" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="N31" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="O31" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P31" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q31" s="4" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="R31" s="4" t="inlineStr">
         <is>
-          <t>styczeń (nowe stawki)</t>
+          <t>cały rok</t>
         </is>
       </c>
       <c r="S31" s="4" t="inlineStr">
@@ -3830,47 +3830,47 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Taryfy i ceny prądu</t>
+          <t>Rachunek za prąd i opłaty</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Koniec mrożenia cen prądu: co zmieniło się w rachunkach w 2026 r.</t>
+          <t>Opłata mocowa: kto płaci, ile i dlaczego</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>mrożenie cen prądu</t>
+          <t>opłata mocowa</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>mrożenie cen prądu 2026; koniec mrożenia cen; ceny prądu od stycznia 2026</t>
+          <t>opłata mocowa 2026; opłata mocowa co to; opłata mocowa stawki</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>informacyjna</t>
+          <t>porównawcza</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>dom</t>
+          <t>wszyscy</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/koniec-mrozenia-cen-pradu</t>
+          <t>/poradniki/oplata-mocowa</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/ceny-pradu</t>
+          <t>/przewodniki/rachunek-za-prad</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>akapit</t>
+          <t>tabela</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr">
@@ -3895,7 +3895,7 @@
       </c>
       <c r="R32" s="4" t="inlineStr">
         <is>
-          <t>grudzień–styczeń</t>
+          <t>styczeń (nowe stawki)</t>
         </is>
       </c>
       <c r="S32" s="4" t="inlineStr">
@@ -3915,67 +3915,67 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>katalog</t>
+          <t>artykuł</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Regiony i operatorzy sieci</t>
+          <t>Taryfy i ceny prądu</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Operatorzy sieci w Polsce: kto dostarcza prąd w Twoim regionie</t>
+          <t>Koniec mrożenia cen prądu: co zmieniło się w rachunkach w 2026 r.</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>operator sieci dystrybucyjnej</t>
+          <t>mrożenie cen prądu</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>OSD lista; dystrybutor prądu w moim regionie; mapa operatorów</t>
+          <t>mrożenie cen prądu 2026; koniec mrożenia cen; ceny prądu od stycznia 2026</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>informacyjna i nawigacyjna</t>
+          <t>informacyjna</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>wszyscy</t>
+          <t>dom</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>/operatorzy</t>
+          <t>/poradniki/koniec-mrozenia-cen-pradu</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>/regiony</t>
+          <t>/przewodniki/ceny-pradu</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>tabela</t>
+          <t>akapit</t>
         </is>
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>CollectionPage + ItemList + BreadcrumbList</t>
+          <t>Article + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M33" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N33" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O33" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P33" s="4" t="n">
         <v>2</v>
@@ -3985,12 +3985,12 @@
       </c>
       <c r="R33" s="4" t="inlineStr">
         <is>
-          <t>cały rok</t>
+          <t>grudzień–styczeń</t>
         </is>
       </c>
       <c r="S33" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 20.11)</t>
         </is>
       </c>
       <c r="T33" s="4" t="inlineStr">
@@ -4005,7 +4005,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>profil operatora</t>
+          <t>katalog</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -4015,22 +4015,22 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>PGE Dystrybucja: taryfa dystrybucyjna, awarie, przyłącza i kontakt</t>
+          <t>Operatorzy sieci w Polsce: kto dostarcza prąd w Twoim regionie</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>PGE Dystrybucja</t>
+          <t>operator sieci dystrybucyjnej</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>PGE Dystrybucja awaria; PGE Dystrybucja wyłączenia prądu; PGE Dystrybucja przyłącze; PGE Dystrybucja taryfa 2027</t>
+          <t>OSD lista; dystrybutor prądu w moim regionie; mapa operatorów</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>nawigacyjna i informacyjna</t>
+          <t>informacyjna i nawigacyjna</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>/operatorzy/pge-dystrybucja</t>
+          <t>/operatorzy</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -4055,7 +4055,7 @@
       </c>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>WebPage (about: Organization) + BreadcrumbList</t>
+          <t>CollectionPage + ItemList + BreadcrumbList</t>
         </is>
       </c>
       <c r="M34" s="4" t="n">
@@ -4075,7 +4075,7 @@
       </c>
       <c r="R34" s="4" t="inlineStr">
         <is>
-          <t>awarie: zima, burze letnie</t>
+          <t>cały rok</t>
         </is>
       </c>
       <c r="S34" s="4" t="inlineStr">
@@ -4105,17 +4105,17 @@
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>TAURON Dystrybucja: taryfa dystrybucyjna, awarie, przyłącza i kontakt</t>
+          <t>PGE Dystrybucja: taryfa dystrybucyjna, awarie, przyłącza i kontakt</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>TAURON Dystrybucja</t>
+          <t>PGE Dystrybucja</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>TAURON Dystrybucja awaria; TAURON Dystrybucja wyłączenia prądu; TAURON Dystrybucja przyłącze; TAURON Dystrybucja taryfa 2027</t>
+          <t>PGE Dystrybucja awaria; PGE Dystrybucja wyłączenia prądu; PGE Dystrybucja przyłącze; PGE Dystrybucja taryfa 2027</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -4130,7 +4130,7 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>/operatorzy/tauron-dystrybucja</t>
+          <t>/operatorzy/pge-dystrybucja</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -4195,17 +4195,17 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Enea Operator: taryfa dystrybucyjna, awarie, przyłącza i kontakt</t>
+          <t>TAURON Dystrybucja: taryfa dystrybucyjna, awarie, przyłącza i kontakt</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Enea Operator</t>
+          <t>TAURON Dystrybucja</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Enea Operator awaria; Enea Operator wyłączenia prądu; Enea Operator przyłącze; Enea Operator taryfa 2027</t>
+          <t>TAURON Dystrybucja awaria; TAURON Dystrybucja wyłączenia prądu; TAURON Dystrybucja przyłącze; TAURON Dystrybucja taryfa 2027</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -4220,7 +4220,7 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>/operatorzy/enea-operator</t>
+          <t>/operatorzy/tauron-dystrybucja</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -4285,17 +4285,17 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Energa-Operator: taryfa dystrybucyjna, awarie, przyłącza i kontakt</t>
+          <t>Enea Operator: taryfa dystrybucyjna, awarie, przyłącza i kontakt</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>Energa-Operator</t>
+          <t>Enea Operator</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Energa-Operator awaria; Energa-Operator wyłączenia prądu; Energa-Operator przyłącze; Energa-Operator taryfa 2027</t>
+          <t>Enea Operator awaria; Enea Operator wyłączenia prądu; Enea Operator przyłącze; Enea Operator taryfa 2027</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>/operatorzy/energa-operator</t>
+          <t>/operatorzy/enea-operator</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -4375,17 +4375,17 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Stoen Operator: taryfa dystrybucyjna, awarie, przyłącza i kontakt</t>
+          <t>Energa-Operator: taryfa dystrybucyjna, awarie, przyłącza i kontakt</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Stoen Operator</t>
+          <t>Energa-Operator</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Stoen Operator awaria; Stoen Operator wyłączenia prądu; Stoen Operator przyłącze; Stoen Operator taryfa 2027</t>
+          <t>Energa-Operator awaria; Energa-Operator wyłączenia prądu; Energa-Operator przyłącze; Energa-Operator taryfa 2027</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>/operatorzy/stoen-operator</t>
+          <t>/operatorzy/energa-operator</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -4455,32 +4455,32 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>tracker</t>
+          <t>profil operatora</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Umowy i zmiana sprzedawcy</t>
+          <t>Regiony i operatorzy sieci</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>CSIRE i zmiana sprzedawcy w 24 godziny: stan wdrożenia</t>
+          <t>Stoen Operator: taryfa dystrybucyjna, awarie, przyłącza i kontakt</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>CSIRE</t>
+          <t>Stoen Operator</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>co to jest CSIRE; zmiana sprzedawcy w 24 godziny; CSIRE termin; mojeIRE</t>
+          <t>Stoen Operator awaria; Stoen Operator wyłączenia prądu; Stoen Operator przyłącze; Stoen Operator taryfa 2027</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>informacyjna (świeżość)</t>
+          <t>nawigacyjna i informacyjna</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
@@ -4490,26 +4490,26 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>/na-biezaco/csire</t>
+          <t>/operatorzy/stoen-operator</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
+          <t>/regiony</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>tabela</t>
         </is>
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>NewsArticle (aktualizowany) + BreadcrumbList</t>
+          <t>WebPage (about: Organization) + BreadcrumbList</t>
         </is>
       </c>
       <c r="M39" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N39" s="4" t="n">
         <v>2</v>
@@ -4518,24 +4518,24 @@
         <v>3</v>
       </c>
       <c r="P39" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q39" s="4" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="R39" s="4" t="inlineStr">
         <is>
-          <t>październik 2026 i kolejne miesiące</t>
+          <t>awarie: zima, burze letnie</t>
         </is>
       </c>
       <c r="S39" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 2 (do 4.12)</t>
         </is>
       </c>
       <c r="T39" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: temat świeży (termin 19.10.2026), poradniki o mojeIRE w mediach branżowych (globenergia.pl). | Brak wolumenu. Sygnał: 45 891 zmian sprzedawcy prądu w I półroczu 2026 r. (URE).</t>
+          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
         </is>
       </c>
     </row>
@@ -4545,77 +4545,77 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>artykuł</t>
+          <t>tracker</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Taryfy i ceny prądu</t>
+          <t>Umowy i zmiana sprzedawcy</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>G11 czy G12: kiedy taryfa dwustrefowa się opłaca</t>
+          <t>CSIRE i zmiana sprzedawcy w 24 godziny: stan wdrożenia</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>taryfa G12</t>
+          <t>CSIRE</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>G11 czy G12; taryfa G12 godziny; taryfa G12w; kiedy opłaca się G12</t>
+          <t>co to jest CSIRE; zmiana sprzedawcy w 24 godziny; CSIRE termin; mojeIRE</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>porównawcza</t>
+          <t>informacyjna (świeżość)</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>dom</t>
+          <t>wszyscy</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/g11-czy-g12</t>
+          <t>/na-biezaco/csire</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/ceny-pradu</t>
+          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
         </is>
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>tabela</t>
+          <t>lista</t>
         </is>
       </c>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>Article + BreadcrumbList + FAQPage</t>
+          <t>NewsArticle (aktualizowany) + BreadcrumbList</t>
         </is>
       </c>
       <c r="M40" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N40" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O40" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="N40" s="4" t="n">
+      <c r="P40" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="O40" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P40" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="Q40" s="4" t="n">
         <v>18</v>
       </c>
       <c r="R40" s="4" t="inlineStr">
         <is>
-          <t>cały rok</t>
+          <t>październik 2026 i kolejne miesiące</t>
         </is>
       </c>
       <c r="S40" s="4" t="inlineStr">
@@ -4625,7 +4625,7 @@
       </c>
       <c r="T40" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: liczne poradniki G11 czy G12 publikowane w 2026 r.</t>
+          <t>Brak wolumenu. Sygnał: temat świeży (termin 19.10.2026), poradniki o mojeIRE w mediach branżowych (globenergia.pl). | Brak wolumenu. Sygnał: 45 891 zmian sprzedawcy prądu w I półroczu 2026 r. (URE).</t>
         </is>
       </c>
     </row>
@@ -4640,47 +4640,47 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Energia dla firm</t>
+          <t>Taryfy i ceny prądu</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Z czego składa się cena prądu dla firm</t>
+          <t>G11 czy G12: kiedy taryfa dwustrefowa się opłaca</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>cena prądu dla firm składniki</t>
+          <t>taryfa G12</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>opłaty na fakturze za prąd w firmie; dystrybucja dla firm; taryfa C11</t>
+          <t>G11 czy G12; taryfa G12 godziny; taryfa G12w; kiedy opłaca się G12</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>informacyjna</t>
+          <t>porównawcza</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>mikro, msp</t>
+          <t>dom</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/cena-pradu-dla-firm-skladniki</t>
+          <t>/poradniki/g11-czy-g12</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/prad-dla-firm</t>
+          <t>/przewodniki/ceny-pradu</t>
         </is>
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>tabela</t>
         </is>
       </c>
       <c r="L41" s="4" t="inlineStr">
@@ -4689,13 +4689,13 @@
         </is>
       </c>
       <c r="M41" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N41" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O41" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P41" s="4" t="n">
         <v>1</v>
@@ -4710,12 +4710,12 @@
       </c>
       <c r="S41" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 20.11)</t>
         </is>
       </c>
       <c r="T41" s="4" t="inlineStr">
         <is>
-          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
+          <t>Brak wolumenu. Sygnał: liczne poradniki G11 czy G12 publikowane w 2026 r.</t>
         </is>
       </c>
     </row>
@@ -4730,22 +4730,22 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Umowy i zmiana sprzedawcy</t>
+          <t>Energia dla firm</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Umowa na prąd: 10 zapisów, które trzeba sprawdzić</t>
+          <t>Z czego składa się cena prądu dla firm</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>umowa na prąd</t>
+          <t>cena prądu dla firm składniki</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>na co uważać w umowie na prąd; opłata handlowa; automatyczne przedłużenie umowy</t>
+          <t>opłaty na fakturze za prąd w firmie; dystrybucja dla firm; taryfa C11</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -4755,17 +4755,17 @@
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>dom, mikro</t>
+          <t>mikro, msp</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/umowa-na-prad-co-sprawdzic</t>
+          <t>/poradniki/cena-pradu-dla-firm-skladniki</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
+          <t>/przewodniki/prad-dla-firm</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
@@ -4820,22 +4820,22 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Samorządy i społeczności energetyczne</t>
+          <t>Umowy i zmiana sprzedawcy</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Jak samorządy kupują energię: przetargi grupowe</t>
+          <t>Umowa na prąd: 10 zapisów, które trzeba sprawdzić</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>przetarg na energię dla gminy</t>
+          <t>umowa na prąd</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>zakup energii przez gminę; grupa zakupowa energii; PZP energia</t>
+          <t>na co uważać w umowie na prąd; opłata handlowa; automatyczne przedłużenie umowy</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -4845,17 +4845,17 @@
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>samorządy</t>
+          <t>dom, mikro</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/przetarg-na-energie-dla-gminy</t>
+          <t>/poradniki/umowa-na-prad-co-sprawdzic</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/energia-dla-samorzadow</t>
+          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
         </is>
       </c>
       <c r="K43" s="4" t="inlineStr">
@@ -4869,7 +4869,7 @@
         </is>
       </c>
       <c r="M43" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N43" s="4" t="n">
         <v>3</v>
@@ -4878,14 +4878,14 @@
         <v>3</v>
       </c>
       <c r="P43" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q43" s="4" t="n">
         <v>18</v>
       </c>
       <c r="R43" s="4" t="inlineStr">
         <is>
-          <t>III–IV kwartał</t>
+          <t>cały rok</t>
         </is>
       </c>
       <c r="S43" s="4" t="inlineStr">
@@ -4905,47 +4905,47 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>poradnik</t>
+          <t>artykuł</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Rachunek za prąd i opłaty</t>
+          <t>Samorządy i społeczności energetyczne</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Jak złożyć reklamację rachunku za prąd</t>
+          <t>Jak samorządy kupują energię: przetargi grupowe</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>reklamacja rachunku za prąd</t>
+          <t>przetarg na energię dla gminy</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>reklamacja faktury za prąd wzór; zawyżony rachunek za prąd</t>
+          <t>zakup energii przez gminę; grupa zakupowa energii; PZP energia</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>poradnikowa (jak)</t>
+          <t>informacyjna</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>dom, mikro</t>
+          <t>samorządy</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/reklamacja-rachunku-za-prad</t>
+          <t>/poradniki/przetarg-na-energie-dla-gminy</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/rachunek-za-prad</t>
+          <t>/przewodniki/energia-dla-samorzadow</t>
         </is>
       </c>
       <c r="K44" s="4" t="inlineStr">
@@ -4955,11 +4955,11 @@
       </c>
       <c r="L44" s="4" t="inlineStr">
         <is>
-          <t>Article (HowTo jako struktura treści) + BreadcrumbList + FAQPage</t>
+          <t>Article + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M44" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N44" s="4" t="n">
         <v>3</v>
@@ -4968,24 +4968,24 @@
         <v>3</v>
       </c>
       <c r="P44" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q44" s="4" t="n">
         <v>18</v>
       </c>
       <c r="R44" s="4" t="inlineStr">
         <is>
-          <t>cały rok</t>
+          <t>III–IV kwartał</t>
         </is>
       </c>
       <c r="S44" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 2 (do 4.12)</t>
         </is>
       </c>
       <c r="T44" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: URE wskazuje pytanie o opłaty na rachunku jako jedno z najczęściej zadawanych (FAQ URE); koniec mrożenia cen od 1.01.2026.</t>
+          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
         </is>
       </c>
     </row>
@@ -5000,22 +5000,22 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Umowy i zmiana sprzedawcy</t>
+          <t>Rachunek za prąd i opłaty</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Jak odstąpić od umowy na prąd podpisanej z akwizytorem</t>
+          <t>Jak złożyć reklamację rachunku za prąd</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>odstąpienie od umowy na prąd</t>
+          <t>reklamacja rachunku za prąd</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>odstąpienie od umowy z akwizytorem; 14 dni na odstąpienie umowa prąd</t>
+          <t>reklamacja faktury za prąd wzór; zawyżony rachunek za prąd</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -5030,12 +5030,12 @@
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/odstapienie-od-umowy-na-prad</t>
+          <t>/poradniki/reklamacja-rachunku-za-prad</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
+          <t>/przewodniki/rachunek-za-prad</t>
         </is>
       </c>
       <c r="K45" s="4" t="inlineStr">
@@ -5075,7 +5075,7 @@
       </c>
       <c r="T45" s="4" t="inlineStr">
         <is>
-          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
+          <t>Brak wolumenu. Sygnał: URE wskazuje pytanie o opłaty na rachunku jako jedno z najczęściej zadawanych (FAQ URE); koniec mrożenia cen od 1.01.2026.</t>
         </is>
       </c>
     </row>
@@ -5095,17 +5095,17 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Jak wypowiedzieć umowę na prąd</t>
+          <t>Jak odstąpić od umowy na prąd podpisanej z akwizytorem</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>wypowiedzenie umowy na prąd</t>
+          <t>odstąpienie od umowy na prąd</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>wypowiedzenie umowy na prąd wzór; okres wypowiedzenia umowy na prąd</t>
+          <t>odstąpienie od umowy z akwizytorem; 14 dni na odstąpienie umowa prąd</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -5120,7 +5120,7 @@
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/wypowiedzenie-umowy-na-prad</t>
+          <t>/poradniki/odstapienie-od-umowy-na-prad</t>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr">
@@ -5180,22 +5180,22 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Energia dla firm</t>
+          <t>Umowy i zmiana sprzedawcy</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>Jak wypowiedzieć umowę na prąd w firmie</t>
+          <t>Jak wypowiedzieć umowę na prąd</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>wypowiedzenie umowy na prąd firma</t>
+          <t>wypowiedzenie umowy na prąd</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>kara za zerwanie umowy na prąd firma</t>
+          <t>wypowiedzenie umowy na prąd wzór; okres wypowiedzenia umowy na prąd</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -5205,17 +5205,17 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>msp</t>
+          <t>dom, mikro</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/wypowiedzenie-umowy-na-prad-firma</t>
+          <t>/poradniki/wypowiedzenie-umowy-na-prad</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/prad-dla-firm</t>
+          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
         </is>
       </c>
       <c r="K47" s="4" t="inlineStr">
@@ -5229,7 +5229,7 @@
         </is>
       </c>
       <c r="M47" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N47" s="4" t="n">
         <v>3</v>
@@ -5238,7 +5238,7 @@
         <v>3</v>
       </c>
       <c r="P47" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q47" s="4" t="n">
         <v>18</v>
@@ -5250,7 +5250,7 @@
       </c>
       <c r="S47" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 20.11)</t>
         </is>
       </c>
       <c r="T47" s="4" t="inlineStr">
@@ -5270,22 +5270,22 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Taryfy i ceny prądu</t>
+          <t>Energia dla firm</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Jak przejść na umowę z ceną dynamiczną</t>
+          <t>Jak wypowiedzieć umowę na prąd w firmie</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>jak przejść na taryfę dynamiczną</t>
+          <t>wypowiedzenie umowy na prąd firma</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>umowa z ceną dynamiczną jak zawrzeć; licznik zdalnego odczytu taryfa dynamiczna</t>
+          <t>kara za zerwanie umowy na prąd firma</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -5295,17 +5295,17 @@
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>dom, mikro</t>
+          <t>msp</t>
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/jak-przejsc-na-taryfe-dynamiczna</t>
+          <t>/poradniki/wypowiedzenie-umowy-na-prad-firma</t>
         </is>
       </c>
       <c r="J48" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/ceny-pradu</t>
+          <t>/przewodniki/prad-dla-firm</t>
         </is>
       </c>
       <c r="K48" s="4" t="inlineStr">
@@ -5345,7 +5345,7 @@
       </c>
       <c r="T48" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: 4 836 gospodarstw domowych z ceną dynamiczną na koniec 2025 r. wobec 135 rok wcześniej; liczniki zdalnego odczytu u 48% odbiorców (URE).</t>
+          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
         </is>
       </c>
     </row>
@@ -5355,28 +5355,32 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>wzór pisma</t>
+          <t>poradnik</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Umowy i zmiana sprzedawcy</t>
+          <t>Taryfy i ceny prądu</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Wzór oświadczenia o odstąpieniu od umowy na prąd</t>
+          <t>Jak przejść na umowę z ceną dynamiczną</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>odstąpienie od umowy wzór</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr"/>
+          <t>jak przejść na taryfę dynamiczną</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>umowa z ceną dynamiczną jak zawrzeć; licznik zdalnego odczytu taryfa dynamiczna</t>
+        </is>
+      </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>transakcyjna (pobranie)</t>
+          <t>poradnikowa (jak)</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
@@ -5386,12 +5390,12 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>/wzory-pism/odstapienie-od-umowy-na-prad</t>
+          <t>/poradniki/jak-przejsc-na-taryfe-dynamiczna</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
+          <t>/przewodniki/ceny-pradu</t>
         </is>
       </c>
       <c r="K49" s="4" t="inlineStr">
@@ -5401,11 +5405,11 @@
       </c>
       <c r="L49" s="4" t="inlineStr">
         <is>
-          <t>Article + DigitalDocument + BreadcrumbList</t>
+          <t>Article (HowTo jako struktura treści) + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M49" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N49" s="4" t="n">
         <v>3</v>
@@ -5414,7 +5418,7 @@
         <v>3</v>
       </c>
       <c r="P49" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q49" s="4" t="n">
         <v>18</v>
@@ -5431,7 +5435,7 @@
       </c>
       <c r="T49" s="4" t="inlineStr">
         <is>
-          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
+          <t>Brak wolumenu. Sygnał: 4 836 gospodarstw domowych z ceną dynamiczną na koniec 2025 r. wobec 135 rok wcześniej; liczniki zdalnego odczytu u 48% odbiorców (URE).</t>
         </is>
       </c>
     </row>
@@ -5451,12 +5455,12 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Wzór wypowiedzenia umowy sprzedaży energii</t>
+          <t>Wzór oświadczenia o odstąpieniu od umowy na prąd</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>wypowiedzenie umowy na prąd wzór</t>
+          <t>odstąpienie od umowy wzór</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr"/>
@@ -5472,7 +5476,7 @@
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>/wzory-pism/wypowiedzenie-umowy-na-prad</t>
+          <t>/wzory-pism/odstapienie-od-umowy-na-prad</t>
         </is>
       </c>
       <c r="J50" s="4" t="inlineStr">
@@ -5537,12 +5541,12 @@
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Wzór reklamacji rachunku za prąd</t>
+          <t>Wzór wypowiedzenia umowy sprzedaży energii</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>reklamacja rachunku za prąd wzór</t>
+          <t>wypowiedzenie umowy na prąd wzór</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr"/>
@@ -5558,7 +5562,7 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>/wzory-pism/reklamacja-rachunku-za-prad</t>
+          <t>/wzory-pism/wypowiedzenie-umowy-na-prad</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr">
@@ -5618,17 +5622,17 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Taryfy i ceny prądu</t>
+          <t>Umowy i zmiana sprzedawcy</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Wzór wniosku o zmianę grupy taryfowej</t>
+          <t>Wzór reklamacji rachunku za prąd</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>wniosek o zmianę taryfy wzór</t>
+          <t>reklamacja rachunku za prąd wzór</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr"/>
@@ -5644,12 +5648,12 @@
       </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>/wzory-pism/zmiana-grupy-taryfowej</t>
+          <t>/wzory-pism/reklamacja-rachunku-za-prad</t>
         </is>
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/ceny-pradu</t>
+          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
         </is>
       </c>
       <c r="K52" s="4" t="inlineStr">
@@ -5704,17 +5708,17 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Umowy i zmiana sprzedawcy</t>
+          <t>Taryfy i ceny prądu</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Wzór wniosku o bonifikatę za przerwę w dostawie energii</t>
+          <t>Wzór wniosku o zmianę grupy taryfowej</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>bonifikata za brak prądu wzór</t>
+          <t>wniosek o zmianę taryfy wzór</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr"/>
@@ -5730,12 +5734,12 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>/wzory-pism/bonifikata-za-przerwe-w-dostawie</t>
+          <t>/wzory-pism/zmiana-grupy-taryfowej</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
+          <t>/przewodniki/ceny-pradu</t>
         </is>
       </c>
       <c r="K53" s="4" t="inlineStr">
@@ -5785,64 +5789,60 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>artykuł</t>
+          <t>wzór pisma</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Rynek i system energetyczny</t>
+          <t>Umowy i zmiana sprzedawcy</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Ujemne ceny prądu: co oznaczają dla odbiorców</t>
+          <t>Wzór wniosku o bonifikatę za przerwę w dostawie energii</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>ujemne ceny prądu</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
-        <is>
-          <t>ceny ujemne energii; dlaczego cena prądu jest ujemna; czy płacą za zużycie prądu</t>
-        </is>
-      </c>
+          <t>bonifikata za brak prądu wzór</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr"/>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>informacyjna</t>
+          <t>transakcyjna (pobranie)</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>dom, firmy</t>
+          <t>dom, mikro</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/ujemne-ceny-pradu</t>
+          <t>/wzory-pism/bonifikata-za-przerwe-w-dostawie</t>
         </is>
       </c>
       <c r="J54" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/rynek-energii</t>
+          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
         </is>
       </c>
       <c r="K54" s="4" t="inlineStr">
         <is>
-          <t>akapit</t>
+          <t>lista</t>
         </is>
       </c>
       <c r="L54" s="4" t="inlineStr">
         <is>
-          <t>Article + BreadcrumbList + FAQPage</t>
+          <t>Article + DigitalDocument + BreadcrumbList</t>
         </is>
       </c>
       <c r="M54" s="4" t="n">
         <v>2</v>
       </c>
       <c r="N54" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O54" s="4" t="n">
         <v>3</v>
@@ -5851,11 +5851,11 @@
         <v>1</v>
       </c>
       <c r="Q54" s="4" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="R54" s="4" t="inlineStr">
         <is>
-          <t>kwiecień–sierpień</t>
+          <t>cały rok</t>
         </is>
       </c>
       <c r="S54" s="4" t="inlineStr">
@@ -5875,57 +5875,57 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>poradnik</t>
+          <t>artykuł</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Taryfy i ceny prądu</t>
+          <t>Rynek i system energetyczny</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Jak zmienić taryfę z G11 na G12</t>
+          <t>Ujemne ceny prądu: co oznaczają dla odbiorców</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>zmiana taryfy G11 na G12</t>
+          <t>ujemne ceny prądu</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>jak zmienić taryfę na G12; wniosek o zmianę taryfy</t>
+          <t>ceny ujemne energii; dlaczego cena prądu jest ujemna; czy płacą za zużycie prądu</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>poradnikowa (jak)</t>
+          <t>informacyjna</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>dom, mikro</t>
+          <t>dom, firmy</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/zmiana-taryfy-G11-na-G12</t>
+          <t>/poradniki/ujemne-ceny-pradu</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/ceny-pradu</t>
+          <t>/przewodniki/rynek-energii</t>
         </is>
       </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>akapit</t>
         </is>
       </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>Article (HowTo jako struktura treści) + BreadcrumbList + FAQPage</t>
+          <t>Article + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M55" s="4" t="n">
@@ -5945,17 +5945,17 @@
       </c>
       <c r="R55" s="4" t="inlineStr">
         <is>
-          <t>cały rok</t>
+          <t>kwiecień–sierpień</t>
         </is>
       </c>
       <c r="S55" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 2 (do 4.12)</t>
         </is>
       </c>
       <c r="T55" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: liczne poradniki G11 czy G12 publikowane w 2026 r.</t>
+          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
         </is>
       </c>
     </row>
@@ -5970,22 +5970,22 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Regiony i operatorzy sieci</t>
+          <t>Taryfy i ceny prądu</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Jak sprawdzić, kto jest Twoim operatorem sieci</t>
+          <t>Jak zmienić taryfę z G11 na G12</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>operator sieci dystrybucyjnej</t>
+          <t>zmiana taryfy G11 na G12</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>jaki mam operator prądu; OSD w mojej okolicy</t>
+          <t>jak zmienić taryfę na G12; wniosek o zmianę taryfy</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
@@ -6000,12 +6000,12 @@
       </c>
       <c r="I56" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/operator-sieci-dystrybucyjnej</t>
+          <t>/poradniki/zmiana-taryfy-G11-na-G12</t>
         </is>
       </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
-          <t>/regiony</t>
+          <t>/przewodniki/ceny-pradu</t>
         </is>
       </c>
       <c r="K56" s="4" t="inlineStr">
@@ -6045,7 +6045,7 @@
       </c>
       <c r="T56" s="4" t="inlineStr">
         <is>
-          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
+          <t>Brak wolumenu. Sygnał: liczne poradniki G11 czy G12 publikowane w 2026 r.</t>
         </is>
       </c>
     </row>
@@ -6060,22 +6060,22 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Umowy i zmiana sprzedawcy</t>
+          <t>Regiony i operatorzy sieci</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Jak przepisać prąd przy przeprowadzce lub zakupie mieszkania</t>
+          <t>Jak sprawdzić, kto jest Twoim operatorem sieci</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>przepisanie licznika prądu</t>
+          <t>operator sieci dystrybucyjnej</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>jak przepisać licznik na siebie; umowa na prąd nowe mieszkanie</t>
+          <t>jaki mam operator prądu; OSD w mojej okolicy</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -6090,12 +6090,12 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/przepisanie-licznika-pradu</t>
+          <t>/poradniki/operator-sieci-dystrybucyjnej</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
+          <t>/regiony</t>
         </is>
       </c>
       <c r="K57" s="4" t="inlineStr">
@@ -6130,7 +6130,7 @@
       </c>
       <c r="S57" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 20.11)</t>
         </is>
       </c>
       <c r="T57" s="4" t="inlineStr">
@@ -6150,22 +6150,22 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Regiony i operatorzy sieci</t>
+          <t>Umowy i zmiana sprzedawcy</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Jak przyłączyć dom do sieci elektroenergetycznej</t>
+          <t>Jak przepisać prąd przy przeprowadzce lub zakupie mieszkania</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>przyłącze prądu</t>
+          <t>przepisanie licznika prądu</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>warunki przyłączenia; ile kosztuje przyłącze prądu; jak długo czeka się na przyłącze</t>
+          <t>jak przepisać licznik na siebie; umowa na prąd nowe mieszkanie</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
@@ -6180,12 +6180,12 @@
       </c>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/przylacze-pradu</t>
+          <t>/poradniki/przepisanie-licznika-pradu</t>
         </is>
       </c>
       <c r="J58" s="4" t="inlineStr">
         <is>
-          <t>/regiony</t>
+          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
         </is>
       </c>
       <c r="K58" s="4" t="inlineStr">
@@ -6240,22 +6240,22 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Rachunek za prąd i opłaty</t>
+          <t>Regiony i operatorzy sieci</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Jak obniżyć rachunek za prąd: sposoby z wyliczeniem oszczędności</t>
+          <t>Jak przyłączyć dom do sieci elektroenergetycznej</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>jak obniżyć rachunek za prąd</t>
+          <t>przyłącze prądu</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>jak oszczędzać prąd; co zużywa najwięcej prądu</t>
+          <t>warunki przyłączenia; ile kosztuje przyłącze prądu; jak długo czeka się na przyłącze</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
@@ -6270,12 +6270,12 @@
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/jak-obnizyc-rachunek-za-prad</t>
+          <t>/poradniki/przylacze-pradu</t>
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/rachunek-za-prad</t>
+          <t>/regiony</t>
         </is>
       </c>
       <c r="K59" s="4" t="inlineStr">
@@ -6289,16 +6289,16 @@
         </is>
       </c>
       <c r="M59" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N59" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O59" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P59" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="P59" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="Q59" s="4" t="n">
         <v>12</v>
@@ -6310,12 +6310,12 @@
       </c>
       <c r="S59" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 2 (do 4.12)</t>
         </is>
       </c>
       <c r="T59" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: URE wskazuje pytanie o opłaty na rachunku jako jedno z najczęściej zadawanych (FAQ URE); koniec mrożenia cen od 1.01.2026.</t>
+          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
         </is>
       </c>
     </row>
@@ -6330,22 +6330,22 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Prosumenci i OZE</t>
+          <t>Rachunek za prąd i opłaty</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>Jak działa depozyt prosumencki i jak czytać rozliczenie</t>
+          <t>Jak obniżyć rachunek za prąd: sposoby z wyliczeniem oszczędności</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>depozyt prosumencki</t>
+          <t>jak obniżyć rachunek za prąd</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>rozliczenie net-billing faktura; zwrot nadpłaty prosument</t>
+          <t>jak oszczędzać prąd; co zużywa najwięcej prądu</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
@@ -6360,12 +6360,12 @@
       </c>
       <c r="I60" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/depozyt-prosumencki</t>
+          <t>/poradniki/jak-obnizyc-rachunek-za-prad</t>
         </is>
       </c>
       <c r="J60" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/fotowoltaika</t>
+          <t>/przewodniki/rachunek-za-prad</t>
         </is>
       </c>
       <c r="K60" s="4" t="inlineStr">
@@ -6379,16 +6379,16 @@
         </is>
       </c>
       <c r="M60" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N60" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O60" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P60" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q60" s="4" t="n">
         <v>12</v>
@@ -6400,12 +6400,12 @@
       </c>
       <c r="S60" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 20.11)</t>
         </is>
       </c>
       <c r="T60" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: temat rozliczeń prosumentów stale wraca w mediach (kb.pl, android.com.pl).</t>
+          <t>Brak wolumenu. Sygnał: URE wskazuje pytanie o opłaty na rachunku jako jedno z najczęściej zadawanych (FAQ URE); koniec mrożenia cen od 1.01.2026.</t>
         </is>
       </c>
     </row>
@@ -6420,22 +6420,22 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Umowy i zmiana sprzedawcy</t>
+          <t>Prosumenci i OZE</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>Co zrobić, gdy grozi wstrzymanie dostaw prądu</t>
+          <t>Jak działa depozyt prosumencki i jak czytać rozliczenie</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>wstrzymanie dostaw prądu</t>
+          <t>depozyt prosumencki</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>odcięcie prądu za długi; wstrzymanie dostaw energii procedura</t>
+          <t>rozliczenie net-billing faktura; zwrot nadpłaty prosument</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
@@ -6450,12 +6450,12 @@
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/wstrzymanie-dostaw-pradu</t>
+          <t>/poradniki/depozyt-prosumencki</t>
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
+          <t>/przewodniki/fotowoltaika</t>
         </is>
       </c>
       <c r="K61" s="4" t="inlineStr">
@@ -6495,7 +6495,7 @@
       </c>
       <c r="T61" s="4" t="inlineStr">
         <is>
-          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
+          <t>Brak wolumenu. Sygnał: temat rozliczeń prosumentów stale wraca w mediach (kb.pl, android.com.pl).</t>
         </is>
       </c>
     </row>
@@ -6510,22 +6510,22 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Regiony i operatorzy sieci</t>
+          <t>Umowy i zmiana sprzedawcy</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Jak zgłosić awarię prądu i uzyskać bonifikatę za przerwę</t>
+          <t>Co zrobić, gdy grozi wstrzymanie dostaw prądu</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>awaria prądu</t>
+          <t>wstrzymanie dostaw prądu</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>brak prądu gdzie zgłosić; bonifikata za przerwę w dostawie prądu</t>
+          <t>odcięcie prądu za długi; wstrzymanie dostaw energii procedura</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -6540,12 +6540,12 @@
       </c>
       <c r="I62" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/awaria-pradu</t>
+          <t>/poradniki/wstrzymanie-dostaw-pradu</t>
         </is>
       </c>
       <c r="J62" s="4" t="inlineStr">
         <is>
-          <t>/regiony</t>
+          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
         </is>
       </c>
       <c r="K62" s="4" t="inlineStr">
@@ -6559,13 +6559,13 @@
         </is>
       </c>
       <c r="M62" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N62" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O62" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P62" s="4" t="n">
         <v>1</v>
@@ -6595,32 +6595,32 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>przewodnik</t>
+          <t>poradnik</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Prosumenci i OZE</t>
+          <t>Regiony i operatorzy sieci</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Fotowoltaika w domu: net-billing, opłacalność i rozliczenia</t>
+          <t>Jak zgłosić awarię prądu i uzyskać bonifikatę za przerwę</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>fotowoltaika</t>
+          <t>awaria prądu</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>czy fotowoltaika się opłaca; net-billing; rozliczenie prosumenta; fotowoltaika z magazynem energii</t>
+          <t>brak prądu gdzie zgłosić; bonifikata za przerwę w dostawie prądu</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>informacyjna i porównawcza</t>
+          <t>poradnikowa (jak)</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
@@ -6630,42 +6630,42 @@
       </c>
       <c r="I63" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/fotowoltaika</t>
+          <t>/poradniki/awaria-pradu</t>
         </is>
       </c>
       <c r="J63" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/fotowoltaika</t>
+          <t>/regiony</t>
         </is>
       </c>
       <c r="K63" s="4" t="inlineStr">
         <is>
-          <t>akapit</t>
+          <t>lista</t>
         </is>
       </c>
       <c r="L63" s="4" t="inlineStr">
         <is>
-          <t>Article + BreadcrumbList + FAQPage</t>
+          <t>Article (HowTo jako struktura treści) + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M63" s="4" t="n">
         <v>3</v>
       </c>
       <c r="N63" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O63" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P63" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q63" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="R63" s="4" t="inlineStr">
         <is>
-          <t>marzec–czerwiec</t>
+          <t>cały rok</t>
         </is>
       </c>
       <c r="S63" s="4" t="inlineStr">
@@ -6675,7 +6675,7 @@
       </c>
       <c r="T63" s="4" t="inlineStr">
         <is>
-          <t>Wolumen: „fotowoltaika” ok. 90 500/mies. (agencjaecho.pl, ok. 2026; podobnie widzialnosc.co.pl). Polska 3. na świecie pod względem zainteresowania fotowoltaiką w Google w latach 2020–2025 (komunikat prasowy, VI 2026, metodologia nieopublikowana). | Wolumen: „magazyn energii” ok. 33 100/mies., wzrost ponad 50% r/r, KD 3/100; „magazyn energii 10kw” 12 100; „magazyn energii 20kwh” 6 600 (agencja widzialnosc.co.pl, Planer słów kluczowych lub DataForSEO, ok. IV 2026). Sygnał: 60% wniosków w Mój Prąd 6.0 dotyczyło magazynów; nabór PME2 od 20.10.2026 (NFOŚiGW, za gramwzielone.pl). | Brak wolumenu. Sygnał: temat rozliczeń prosumentów stale wraca w mediach (kb.pl, android.com.pl).</t>
+          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
         </is>
       </c>
     </row>
@@ -6685,7 +6685,7 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>artykuł</t>
+          <t>przewodnik</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -6695,32 +6695,32 @@
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Net-billing: czy fotowoltaika nadal się opłaca</t>
+          <t>Fotowoltaika w domu: net-billing, opłacalność i rozliczenia</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>net-billing</t>
+          <t>fotowoltaika</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>net-billing opłacalność; net-billing jak działa; rozliczenie net-billing</t>
+          <t>czy fotowoltaika się opłaca; net-billing; rozliczenie prosumenta; fotowoltaika z magazynem energii</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>informacyjna</t>
+          <t>informacyjna i porównawcza</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr">
         <is>
-          <t>dom</t>
+          <t>dom, mikro</t>
         </is>
       </c>
       <c r="I64" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/net-billing-czy-fotowoltaika-sie-oplaca</t>
+          <t>/przewodniki/fotowoltaika</t>
         </is>
       </c>
       <c r="J64" s="4" t="inlineStr">
@@ -6765,7 +6765,7 @@
       </c>
       <c r="T64" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: temat rozliczeń prosumentów stale wraca w mediach (kb.pl, android.com.pl).</t>
+          <t>Wolumen: „fotowoltaika” ok. 90 500/mies. (agencjaecho.pl, ok. 2026; podobnie widzialnosc.co.pl). Polska 3. na świecie pod względem zainteresowania fotowoltaiką w Google w latach 2020–2025 (komunikat prasowy, VI 2026, metodologia nieopublikowana). | Wolumen: „magazyn energii” ok. 33 100/mies., wzrost ponad 50% r/r, KD 3/100; „magazyn energii 10kw” 12 100; „magazyn energii 20kwh” 6 600 (agencja widzialnosc.co.pl, Planer słów kluczowych lub DataForSEO, ok. IV 2026). Sygnał: 60% wniosków w Mój Prąd 6.0 dotyczyło magazynów; nabór PME2 od 20.10.2026 (NFOŚiGW, za gramwzielone.pl). | Brak wolumenu. Sygnał: temat rozliczeń prosumentów stale wraca w mediach (kb.pl, android.com.pl).</t>
         </is>
       </c>
     </row>
@@ -6780,22 +6780,22 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Energia dla firm</t>
+          <t>Prosumenci i OZE</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>Moc umowna: jak nie przepłacać</t>
+          <t>Net-billing: czy fotowoltaika nadal się opłaca</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>moc umowna</t>
+          <t>net-billing</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>przekroczenie mocy umownej; jak zmniejszyć moc umowną; opłata za moc</t>
+          <t>net-billing opłacalność; net-billing jak działa; rozliczenie net-billing</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -6805,17 +6805,17 @@
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>msp</t>
+          <t>dom</t>
         </is>
       </c>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/moc-umowna</t>
+          <t>/poradniki/net-billing-czy-fotowoltaika-sie-oplaca</t>
         </is>
       </c>
       <c r="J65" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/prad-dla-firm</t>
+          <t>/przewodniki/fotowoltaika</t>
         </is>
       </c>
       <c r="K65" s="4" t="inlineStr">
@@ -6829,13 +6829,13 @@
         </is>
       </c>
       <c r="M65" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N65" s="4" t="n">
         <v>3</v>
       </c>
       <c r="O65" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P65" s="4" t="n">
         <v>1</v>
@@ -6845,7 +6845,7 @@
       </c>
       <c r="R65" s="4" t="inlineStr">
         <is>
-          <t>cały rok</t>
+          <t>marzec–czerwiec</t>
         </is>
       </c>
       <c r="S65" s="4" t="inlineStr">
@@ -6855,7 +6855,7 @@
       </c>
       <c r="T65" s="4" t="inlineStr">
         <is>
-          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
+          <t>Brak wolumenu. Sygnał: temat rozliczeń prosumentów stale wraca w mediach (kb.pl, android.com.pl).</t>
         </is>
       </c>
     </row>
@@ -6865,7 +6865,7 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>poradnik</t>
+          <t>artykuł</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -6875,22 +6875,22 @@
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>Jak sprawdzić i zmniejszyć moc umowną w firmie</t>
+          <t>Moc umowna: jak nie przepłacać</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>zmniejszenie mocy umownej</t>
+          <t>moc umowna</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>jak obniżyć moc umowną; analiza mocy umownej</t>
+          <t>przekroczenie mocy umownej; jak zmniejszyć moc umowną; opłata za moc</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>poradnikowa (jak)</t>
+          <t>informacyjna</t>
         </is>
       </c>
       <c r="H66" s="4" t="inlineStr">
@@ -6900,7 +6900,7 @@
       </c>
       <c r="I66" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/zmniejszenie-mocy-umownej</t>
+          <t>/poradniki/moc-umowna</t>
         </is>
       </c>
       <c r="J66" s="4" t="inlineStr">
@@ -6910,12 +6910,12 @@
       </c>
       <c r="K66" s="4" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>akapit</t>
         </is>
       </c>
       <c r="L66" s="4" t="inlineStr">
         <is>
-          <t>Article (HowTo jako struktura treści) + BreadcrumbList + FAQPage</t>
+          <t>Article + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M66" s="4" t="n">
@@ -6965,17 +6965,17 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Jak uniknąć opłat za energię bierną</t>
+          <t>Jak sprawdzić i zmniejszyć moc umowną w firmie</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>energia bierna</t>
+          <t>zmniejszenie mocy umownej</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>opłata za energię bierną; kompensacja mocy biernej</t>
+          <t>jak obniżyć moc umowną; analiza mocy umownej</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
@@ -6990,7 +6990,7 @@
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/energia-bierna</t>
+          <t>/poradniki/zmniejszenie-mocy-umownej</t>
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr">
@@ -7045,73 +7045,73 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>artykuł</t>
+          <t>poradnik</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Magazyny, pompy ciepła, samochody elektryczne</t>
+          <t>Energia dla firm</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>Ładowanie samochodu elektrycznego w domu: koszt 100 km</t>
+          <t>Jak uniknąć opłat za energię bierną</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>koszt ładowania samochodu elektrycznego</t>
+          <t>energia bierna</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>ładowanie auta elektrycznego w domu koszt; wallbox; ile kosztuje naładowanie elektryka</t>
+          <t>opłata za energię bierną; kompensacja mocy biernej</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>porównawcza</t>
+          <t>poradnikowa (jak)</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
         <is>
-          <t>dom</t>
+          <t>msp</t>
         </is>
       </c>
       <c r="I68" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/ladowanie-samochodu-elektrycznego-w-domu</t>
+          <t>/poradniki/energia-bierna</t>
         </is>
       </c>
       <c r="J68" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/magazyn-energii</t>
+          <t>/przewodniki/prad-dla-firm</t>
         </is>
       </c>
       <c r="K68" s="4" t="inlineStr">
         <is>
-          <t>tabela</t>
+          <t>lista</t>
         </is>
       </c>
       <c r="L68" s="4" t="inlineStr">
         <is>
-          <t>Article + BreadcrumbList + FAQPage</t>
+          <t>Article (HowTo jako struktura treści) + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M68" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N68" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O68" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P68" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q68" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R68" s="4" t="inlineStr">
         <is>
@@ -7135,57 +7135,57 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>poradnik</t>
+          <t>artykuł</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Rachunek za prąd i opłaty</t>
+          <t>Magazyny, pompy ciepła, samochody elektryczne</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Jak podać odczyt licznika i rozliczyć się według rzeczywistego zużycia</t>
+          <t>Ładowanie samochodu elektrycznego w domu: koszt 100 km</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>odczyt licznika prądu</t>
+          <t>koszt ładowania samochodu elektrycznego</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>jak podać odczyt licznika; samoodczyt licznika</t>
+          <t>ładowanie auta elektrycznego w domu koszt; wallbox; ile kosztuje naładowanie elektryka</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>poradnikowa (jak)</t>
+          <t>porównawcza</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>dom, mikro</t>
+          <t>dom</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/odczyt-licznika-pradu</t>
+          <t>/poradniki/ladowanie-samochodu-elektrycznego-w-domu</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/rachunek-za-prad</t>
+          <t>/przewodniki/magazyn-energii</t>
         </is>
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>tabela</t>
         </is>
       </c>
       <c r="L69" s="4" t="inlineStr">
         <is>
-          <t>Article (HowTo jako struktura treści) + BreadcrumbList + FAQPage</t>
+          <t>Article + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M69" s="4" t="n">
@@ -7230,22 +7230,22 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Prosumenci i OZE</t>
+          <t>Rachunek za prąd i opłaty</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>Jak zostać prosumentem: zgłoszenie mikroinstalacji do operatora</t>
+          <t>Jak podać odczyt licznika i rozliczyć się według rzeczywistego zużycia</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>zgłoszenie mikroinstalacji</t>
+          <t>odczyt licznika prądu</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>jak zostać prosumentem; zgłoszenie fotowoltaiki do OSD</t>
+          <t>jak podać odczyt licznika; samoodczyt licznika</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
@@ -7260,12 +7260,12 @@
       </c>
       <c r="I70" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/zgloszenie-mikroinstalacji</t>
+          <t>/poradniki/odczyt-licznika-pradu</t>
         </is>
       </c>
       <c r="J70" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/fotowoltaika</t>
+          <t>/przewodniki/rachunek-za-prad</t>
         </is>
       </c>
       <c r="K70" s="4" t="inlineStr">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="T70" s="4" t="inlineStr">
         <is>
-          <t>Wolumen: „fotowoltaika” ok. 90 500/mies. (agencjaecho.pl, ok. 2026; podobnie widzialnosc.co.pl). Polska 3. na świecie pod względem zainteresowania fotowoltaiką w Google w latach 2020–2025 (komunikat prasowy, VI 2026, metodologia nieopublikowana).</t>
+          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
         </is>
       </c>
     </row>
@@ -7315,47 +7315,47 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>artykuł</t>
+          <t>poradnik</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Rynek i system energetyczny</t>
+          <t>Prosumenci i OZE</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>Jak działa rynek energii w Polsce: od elektrowni do gniazdka</t>
+          <t>Jak zostać prosumentem: zgłoszenie mikroinstalacji do operatora</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>rynek energii</t>
+          <t>zgłoszenie mikroinstalacji</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>jak działa rynek energii; skąd bierze się cena prądu; TGE</t>
+          <t>jak zostać prosumentem; zgłoszenie fotowoltaiki do OSD</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>informacyjna</t>
+          <t>poradnikowa (jak)</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr">
         <is>
-          <t>wszyscy</t>
+          <t>dom, mikro</t>
         </is>
       </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/jak-dziala-rynek-energii</t>
+          <t>/poradniki/zgloszenie-mikroinstalacji</t>
         </is>
       </c>
       <c r="J71" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/rynek-energii</t>
+          <t>/przewodniki/fotowoltaika</t>
         </is>
       </c>
       <c r="K71" s="4" t="inlineStr">
@@ -7365,23 +7365,23 @@
       </c>
       <c r="L71" s="4" t="inlineStr">
         <is>
-          <t>Article + BreadcrumbList + FAQPage</t>
+          <t>Article (HowTo jako struktura treści) + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M71" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N71" s="4" t="n">
         <v>2</v>
       </c>
       <c r="O71" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q71" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="R71" s="4" t="inlineStr">
         <is>
@@ -7395,7 +7395,7 @@
       </c>
       <c r="T71" s="4" t="inlineStr">
         <is>
-          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
+          <t>Wolumen: „fotowoltaika” ok. 90 500/mies. (agencjaecho.pl, ok. 2026; podobnie widzialnosc.co.pl). Polska 3. na świecie pod względem zainteresowania fotowoltaiką w Google w latach 2020–2025 (komunikat prasowy, VI 2026, metodologia nieopublikowana).</t>
         </is>
       </c>
     </row>
@@ -7410,22 +7410,22 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Umowy i zmiana sprzedawcy</t>
+          <t>Rynek i system energetyczny</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>Sprzedawca rezerwowy: kiedy działa i ile kosztuje</t>
+          <t>Jak działa rynek energii w Polsce: od elektrowni do gniazdka</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>sprzedawca rezerwowy</t>
+          <t>rynek energii</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>sprzedaż rezerwowa; upadłość sprzedawcy energii co dalej</t>
+          <t>jak działa rynek energii; skąd bierze się cena prądu; TGE</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
@@ -7440,17 +7440,17 @@
       </c>
       <c r="I72" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/sprzedawca-rezerwowy</t>
+          <t>/poradniki/jak-dziala-rynek-energii</t>
         </is>
       </c>
       <c r="J72" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
+          <t>/przewodniki/rynek-energii</t>
         </is>
       </c>
       <c r="K72" s="4" t="inlineStr">
         <is>
-          <t>akapit</t>
+          <t>lista</t>
         </is>
       </c>
       <c r="L72" s="4" t="inlineStr">
@@ -7475,7 +7475,7 @@
       </c>
       <c r="R72" s="4" t="inlineStr">
         <is>
-          <t>zdarzeniowa</t>
+          <t>cały rok</t>
         </is>
       </c>
       <c r="S72" s="4" t="inlineStr">
@@ -7485,7 +7485,7 @@
       </c>
       <c r="T72" s="4" t="inlineStr">
         <is>
-          <t>Brak wolumenu. Sygnał: 45 891 zmian sprzedawcy prądu w I półroczu 2026 r. (URE).</t>
+          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
         </is>
       </c>
     </row>
@@ -7495,57 +7495,57 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>poradnik</t>
+          <t>artykuł</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>Regiony i operatorzy sieci</t>
+          <t>Umowy i zmiana sprzedawcy</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>Jak zwiększyć moc przyłączeniową</t>
+          <t>Sprzedawca rezerwowy: kiedy działa i ile kosztuje</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>zwiększenie mocy przyłączeniowej</t>
+          <t>sprzedawca rezerwowy</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>moc przyłączeniowa dom; wniosek o zwiększenie mocy</t>
+          <t>sprzedaż rezerwowa; upadłość sprzedawcy energii co dalej</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>poradnikowa (jak)</t>
+          <t>informacyjna</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
         <is>
-          <t>dom, mikro</t>
+          <t>wszyscy</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/zwiekszenie-mocy-przylaczeniowej</t>
+          <t>/poradniki/sprzedawca-rezerwowy</t>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
         <is>
-          <t>/regiony</t>
+          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
         </is>
       </c>
       <c r="K73" s="4" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>akapit</t>
         </is>
       </c>
       <c r="L73" s="4" t="inlineStr">
         <is>
-          <t>Article (HowTo jako struktura treści) + BreadcrumbList + FAQPage</t>
+          <t>Article + BreadcrumbList + FAQPage</t>
         </is>
       </c>
       <c r="M73" s="4" t="n">
@@ -7565,7 +7565,7 @@
       </c>
       <c r="R73" s="4" t="inlineStr">
         <is>
-          <t>cały rok</t>
+          <t>zdarzeniowa</t>
         </is>
       </c>
       <c r="S73" s="4" t="inlineStr">
@@ -7575,7 +7575,7 @@
       </c>
       <c r="T73" s="4" t="inlineStr">
         <is>
-          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
+          <t>Brak wolumenu. Sygnał: 45 891 zmian sprzedawcy prądu w I półroczu 2026 r. (URE).</t>
         </is>
       </c>
     </row>
@@ -7590,22 +7590,22 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>Samorządy i społeczności energetyczne</t>
+          <t>Regiony i operatorzy sieci</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>Jak założyć spółdzielnię energetyczną</t>
+          <t>Jak zwiększyć moc przyłączeniową</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>spółdzielnia energetyczna</t>
+          <t>zwiększenie mocy przyłączeniowej</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>jak założyć spółdzielnię energetyczną; spółdzielnia energetyczna korzyści</t>
+          <t>moc przyłączeniowa dom; wniosek o zwiększenie mocy</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
@@ -7615,17 +7615,17 @@
       </c>
       <c r="H74" s="4" t="inlineStr">
         <is>
-          <t>samorządy</t>
+          <t>dom, mikro</t>
         </is>
       </c>
       <c r="I74" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/spoldzielnia-energetyczna</t>
+          <t>/poradniki/zwiekszenie-mocy-przylaczeniowej</t>
         </is>
       </c>
       <c r="J74" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/energia-dla-samorzadow</t>
+          <t>/regiony</t>
         </is>
       </c>
       <c r="K74" s="4" t="inlineStr">
@@ -7680,22 +7680,22 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>Umowy i zmiana sprzedawcy</t>
+          <t>Samorządy i społeczności energetyczne</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>Jak złożyć skargę na sprzedawcę lub operatora energii</t>
+          <t>Jak założyć spółdzielnię energetyczną</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>skarga na sprzedawcę energii</t>
+          <t>spółdzielnia energetyczna</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>Rzecznik Odbiorców Paliw i Energii; skarga do URE</t>
+          <t>jak założyć spółdzielnię energetyczną; spółdzielnia energetyczna korzyści</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
@@ -7705,17 +7705,17 @@
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>dom, mikro</t>
+          <t>samorządy</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>/poradniki/skarga-na-sprzedawce-energii</t>
+          <t>/poradniki/spoldzielnia-energetyczna</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
         <is>
-          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
+          <t>/przewodniki/energia-dla-samorzadow</t>
         </is>
       </c>
       <c r="K75" s="4" t="inlineStr">
@@ -7755,12 +7755,102 @@
       </c>
       <c r="T75" s="4" t="inlineStr">
         <is>
+          <t>[DO WERYFIKACJI w narzędziu SEO]</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>poradnik</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Umowy i zmiana sprzedawcy</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Jak złożyć skargę na sprzedawcę lub operatora energii</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>skarga na sprzedawcę energii</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>Rzecznik Odbiorców Paliw i Energii; skarga do URE</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>poradnikowa (jak)</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>dom, mikro</t>
+        </is>
+      </c>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t>/poradniki/skarga-na-sprzedawce-energii</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="inlineStr">
+        <is>
+          <t>/przewodniki/zmiana-sprzedawcy-pradu</t>
+        </is>
+      </c>
+      <c r="K76" s="4" t="inlineStr">
+        <is>
+          <t>lista</t>
+        </is>
+      </c>
+      <c r="L76" s="4" t="inlineStr">
+        <is>
+          <t>Article (HowTo jako struktura treści) + BreadcrumbList + FAQPage</t>
+        </is>
+      </c>
+      <c r="M76" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N76" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O76" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P76" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q76" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R76" s="4" t="inlineStr">
+        <is>
+          <t>cały rok</t>
+        </is>
+      </c>
+      <c r="S76" s="4" t="inlineStr">
+        <is>
+          <t>Fala 2 (do 4.12)</t>
+        </is>
+      </c>
+      <c r="T76" s="4" t="inlineStr">
+        <is>
           <t>Brak wolumenu. Sygnał: 45 891 zmian sprzedawcy prądu w I półroczu 2026 r. (URE).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T75"/>
+  <autoFilter ref="A1:T76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Energypedia: start publiczny 16 listopada 2026 r.
Pakiet startowy, nowy harmonogram MVP i asystenta AI, terminy prac
technicznych i prawnych do 12 XI, fale w mapie tematów.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rv6z9UcN5eHj71s4nzprHT
</commit_message>
<xml_diff>
--- a/docs/energypedia/mapa/Energypedia_mapa_tematow.xlsx
+++ b/docs/energypedia/mapa/Energypedia_mapa_tematow.xlsx
@@ -1220,7 +1220,7 @@
       </c>
       <c r="S2" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T2" s="4" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="S3" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T3" s="4" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="S4" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T4" s="4" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="S5" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T5" s="4" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="S6" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T6" s="4" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="S7" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T7" s="4" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="S8" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T8" s="4" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="S9" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T9" s="4" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="S10" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T10" s="4" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="S11" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T11" s="4" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="S12" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T12" s="4" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="S13" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T13" s="4" t="inlineStr">
@@ -2300,7 +2300,7 @@
       </c>
       <c r="S14" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T14" s="4" t="inlineStr">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T15" s="4" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T16" s="4" t="inlineStr">
@@ -2570,7 +2570,7 @@
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T17" s="4" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T18" s="4" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T19" s="4" t="inlineStr">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="S20" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T20" s="4" t="inlineStr">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="S21" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T21" s="4" t="inlineStr">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="S22" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T22" s="4" t="inlineStr">
@@ -3110,7 +3110,7 @@
       </c>
       <c r="S23" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T23" s="4" t="inlineStr">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="S24" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T24" s="4" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="S25" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T25" s="4" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="S26" s="4" t="inlineStr">
         <is>
-          <t>Tydzień startu</t>
+          <t>Grudzień (Barometr, taryfy)</t>
         </is>
       </c>
       <c r="T26" s="4" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="S27" s="4" t="inlineStr">
         <is>
-          <t>Tydzień startu</t>
+          <t>Grudzień (Barometr, taryfy)</t>
         </is>
       </c>
       <c r="T27" s="4" t="inlineStr">
@@ -3548,7 +3548,7 @@
       </c>
       <c r="S28" s="4" t="inlineStr">
         <is>
-          <t>Tydzień startu</t>
+          <t>Grudzień (Barometr, taryfy)</t>
         </is>
       </c>
       <c r="T28" s="4" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="S29" s="4" t="inlineStr">
         <is>
-          <t>Tydzień startu</t>
+          <t>Grudzień (Barometr, taryfy)</t>
         </is>
       </c>
       <c r="T29" s="4" t="inlineStr">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="S30" s="4" t="inlineStr">
         <is>
-          <t>Tydzień startu</t>
+          <t>Grudzień (Barometr, taryfy)</t>
         </is>
       </c>
       <c r="T30" s="4" t="inlineStr">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="S31" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T31" s="4" t="inlineStr">
@@ -3900,7 +3900,7 @@
       </c>
       <c r="S32" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T32" s="4" t="inlineStr">
@@ -3990,7 +3990,7 @@
       </c>
       <c r="S33" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T33" s="4" t="inlineStr">
@@ -4080,7 +4080,7 @@
       </c>
       <c r="S34" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T34" s="4" t="inlineStr">
@@ -4170,7 +4170,7 @@
       </c>
       <c r="S35" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T35" s="4" t="inlineStr">
@@ -4260,7 +4260,7 @@
       </c>
       <c r="S36" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T36" s="4" t="inlineStr">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="S37" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T37" s="4" t="inlineStr">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="S38" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T38" s="4" t="inlineStr">
@@ -4530,7 +4530,7 @@
       </c>
       <c r="S39" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T39" s="4" t="inlineStr">
@@ -4620,7 +4620,7 @@
       </c>
       <c r="S40" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T40" s="4" t="inlineStr">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="S41" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T41" s="4" t="inlineStr">
@@ -4800,7 +4800,7 @@
       </c>
       <c r="S42" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T42" s="4" t="inlineStr">
@@ -4890,7 +4890,7 @@
       </c>
       <c r="S43" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T43" s="4" t="inlineStr">
@@ -4980,7 +4980,7 @@
       </c>
       <c r="S44" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T44" s="4" t="inlineStr">
@@ -5070,7 +5070,7 @@
       </c>
       <c r="S45" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T45" s="4" t="inlineStr">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="S46" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T46" s="4" t="inlineStr">
@@ -5250,7 +5250,7 @@
       </c>
       <c r="S47" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T47" s="4" t="inlineStr">
@@ -5340,7 +5340,7 @@
       </c>
       <c r="S48" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T48" s="4" t="inlineStr">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="S49" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T49" s="4" t="inlineStr">
@@ -5516,7 +5516,7 @@
       </c>
       <c r="S50" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T50" s="4" t="inlineStr">
@@ -5602,7 +5602,7 @@
       </c>
       <c r="S51" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T51" s="4" t="inlineStr">
@@ -5688,7 +5688,7 @@
       </c>
       <c r="S52" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T52" s="4" t="inlineStr">
@@ -5774,7 +5774,7 @@
       </c>
       <c r="S53" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T53" s="4" t="inlineStr">
@@ -5860,7 +5860,7 @@
       </c>
       <c r="S54" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T54" s="4" t="inlineStr">
@@ -5950,7 +5950,7 @@
       </c>
       <c r="S55" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T55" s="4" t="inlineStr">
@@ -6040,7 +6040,7 @@
       </c>
       <c r="S56" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T56" s="4" t="inlineStr">
@@ -6130,7 +6130,7 @@
       </c>
       <c r="S57" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T57" s="4" t="inlineStr">
@@ -6220,7 +6220,7 @@
       </c>
       <c r="S58" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T58" s="4" t="inlineStr">
@@ -6310,7 +6310,7 @@
       </c>
       <c r="S59" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T59" s="4" t="inlineStr">
@@ -6400,7 +6400,7 @@
       </c>
       <c r="S60" s="4" t="inlineStr">
         <is>
-          <t>Fala 1 (do 20.11)</t>
+          <t>Fala 1 (do 27.11; pakiet startowy do 12.11)</t>
         </is>
       </c>
       <c r="T60" s="4" t="inlineStr">
@@ -6490,7 +6490,7 @@
       </c>
       <c r="S61" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T61" s="4" t="inlineStr">
@@ -6580,7 +6580,7 @@
       </c>
       <c r="S62" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T62" s="4" t="inlineStr">
@@ -6670,7 +6670,7 @@
       </c>
       <c r="S63" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T63" s="4" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="S64" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T64" s="4" t="inlineStr">
@@ -6850,7 +6850,7 @@
       </c>
       <c r="S65" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T65" s="4" t="inlineStr">
@@ -6940,7 +6940,7 @@
       </c>
       <c r="S66" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T66" s="4" t="inlineStr">
@@ -7030,7 +7030,7 @@
       </c>
       <c r="S67" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T67" s="4" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="S68" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T68" s="4" t="inlineStr">
@@ -7210,7 +7210,7 @@
       </c>
       <c r="S69" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T69" s="4" t="inlineStr">
@@ -7300,7 +7300,7 @@
       </c>
       <c r="S70" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T70" s="4" t="inlineStr">
@@ -7390,7 +7390,7 @@
       </c>
       <c r="S71" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T71" s="4" t="inlineStr">
@@ -7480,7 +7480,7 @@
       </c>
       <c r="S72" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T72" s="4" t="inlineStr">
@@ -7570,7 +7570,7 @@
       </c>
       <c r="S73" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T73" s="4" t="inlineStr">
@@ -7660,7 +7660,7 @@
       </c>
       <c r="S74" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T74" s="4" t="inlineStr">
@@ -7750,7 +7750,7 @@
       </c>
       <c r="S75" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T75" s="4" t="inlineStr">
@@ -7840,7 +7840,7 @@
       </c>
       <c r="S76" s="4" t="inlineStr">
         <is>
-          <t>Fala 2 (do 4.12)</t>
+          <t>Fala 2 (do 18.12)</t>
         </is>
       </c>
       <c r="T76" s="4" t="inlineStr">

</xml_diff>